<commit_message>
improved starch absorption kinetics with inhibitors
</commit_message>
<xml_diff>
--- a/meal glucose bread and bread + citric acid.xlsx
+++ b/meal glucose bread and bread + citric acid.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{2047551B-E236-4238-9005-81FCDC5B54B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DE9749A-616F-4E97-ACA3-9235360E8C25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -552,7 +552,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -573,7 +573,6 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
@@ -1179,7 +1178,7 @@
       <c r="D12">
         <v>1</v>
       </c>
-      <c r="E12" s="20">
+      <c r="E12">
         <v>50</v>
       </c>
       <c r="R12"/>
@@ -7880,7 +7879,7 @@
       <c r="G80">
         <v>0</v>
       </c>
-      <c r="H80" s="21">
+      <c r="H80" s="20">
         <v>0</v>
       </c>
       <c r="I80">
@@ -7928,16 +7927,16 @@
       <c r="W80" s="7">
         <v>0</v>
       </c>
-      <c r="X80" s="20">
-        <v>0</v>
-      </c>
-      <c r="Y80" s="20">
-        <v>0</v>
-      </c>
-      <c r="Z80" s="20">
-        <v>0</v>
-      </c>
-      <c r="AA80" s="20">
+      <c r="X80">
+        <v>0</v>
+      </c>
+      <c r="Y80">
+        <v>0</v>
+      </c>
+      <c r="Z80">
+        <v>0</v>
+      </c>
+      <c r="AA80">
         <v>0</v>
       </c>
       <c r="AB80" s="1">
@@ -7981,7 +7980,7 @@
       <c r="G81">
         <v>0</v>
       </c>
-      <c r="H81" s="21">
+      <c r="H81" s="20">
         <v>0</v>
       </c>
       <c r="I81">
@@ -8026,19 +8025,19 @@
       <c r="V81" s="1">
         <v>0</v>
       </c>
-      <c r="W81" s="20">
-        <v>0</v>
-      </c>
-      <c r="X81" s="20">
-        <v>0</v>
-      </c>
-      <c r="Y81" s="20">
-        <v>0</v>
-      </c>
-      <c r="Z81" s="20">
-        <v>0</v>
-      </c>
-      <c r="AA81" s="20">
+      <c r="W81">
+        <v>0</v>
+      </c>
+      <c r="X81">
+        <v>0</v>
+      </c>
+      <c r="Y81">
+        <v>0</v>
+      </c>
+      <c r="Z81">
+        <v>0</v>
+      </c>
+      <c r="AA81">
         <v>0</v>
       </c>
       <c r="AB81" s="1">
@@ -8082,7 +8081,7 @@
       <c r="G82">
         <v>0</v>
       </c>
-      <c r="H82" s="21">
+      <c r="H82" s="20">
         <v>0</v>
       </c>
       <c r="I82">
@@ -8127,19 +8126,19 @@
       <c r="V82" s="1">
         <v>0</v>
       </c>
-      <c r="W82" s="20">
-        <v>0</v>
-      </c>
-      <c r="X82" s="20">
-        <v>0</v>
-      </c>
-      <c r="Y82" s="20">
-        <v>0</v>
-      </c>
-      <c r="Z82" s="20">
-        <v>0</v>
-      </c>
-      <c r="AA82" s="20">
+      <c r="W82">
+        <v>0</v>
+      </c>
+      <c r="X82">
+        <v>0</v>
+      </c>
+      <c r="Y82">
+        <v>0</v>
+      </c>
+      <c r="Z82">
+        <v>0</v>
+      </c>
+      <c r="AA82">
         <v>0</v>
       </c>
       <c r="AB82" s="1">
@@ -8717,7 +8716,7 @@
       <c r="AF87" s="1">
         <v>1.4</v>
       </c>
-      <c r="AG87" s="22">
+      <c r="AG87" s="21">
         <v>1665</v>
       </c>
     </row>

</xml_diff>